<commit_message>
ADD:Cambios de bd Noviembre V2.0
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de sistema/Base de datos/Diccionario de datos BD.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de sistema/Base de datos/Diccionario de datos BD.xlsx
@@ -778,45 +778,45 @@
     <t>firstName</t>
   </si>
   <si>
+    <t>E4FC695C-DB7F-273E-0C47-C01648108DA5</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>914BC5D9-89EB-EF1A-FB0C-E191FFDF845A</t>
+  </si>
+  <si>
+    <t>5F72E1E0-0043-42F1-DBCE-53EE47EBDC8C</t>
+  </si>
+  <si>
+    <t>88D79E68-CA48-4058-D21F-BA79CABB78AB</t>
+  </si>
+  <si>
+    <t>7ABD1485-D415-29B3-802F-B235595EFE87</t>
+  </si>
+  <si>
+    <t>B79CB950-5BF3-4DC8-8B7C-D7770260C2F4</t>
+  </si>
+  <si>
+    <t>56F05333-4945-447A-1128-61D911628D2D</t>
+  </si>
+  <si>
+    <t>72E7BD72-71EA-49B3-00BF-7728CE9660FC</t>
+  </si>
+  <si>
+    <t>96F0A8B5-8BE1-9346-540D-B1A5DB9E97E8</t>
+  </si>
+  <si>
     <t>275B3005-CA60-8E26-87EB-EC4C9886EC39</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>5F72E1E0-0043-42F1-DBCE-53EE47EBDC8C</t>
-  </si>
-  <si>
-    <t>88D79E68-CA48-4058-D21F-BA79CABB78AB</t>
-  </si>
-  <si>
-    <t>E4FC695C-DB7F-273E-0C47-C01648108DA5</t>
-  </si>
-  <si>
-    <t>B79CB950-5BF3-4DC8-8B7C-D7770260C2F4</t>
-  </si>
-  <si>
-    <t>7ABD1485-D415-29B3-802F-B235595EFE87</t>
-  </si>
-  <si>
-    <t>72E7BD72-71EA-49B3-00BF-7728CE9660FC</t>
+    <t>AEC573F9-790B-6348-921B-492CF00715BB</t>
   </si>
   <si>
     <t>0417C238-82AC-A5B2-88E7-F2BB25C183A5</t>
   </si>
   <si>
-    <t>AEC573F9-790B-6348-921B-492CF00715BB</t>
-  </si>
-  <si>
-    <t>96F0A8B5-8BE1-9346-540D-B1A5DB9E97E8</t>
-  </si>
-  <si>
-    <t>914BC5D9-89EB-EF1A-FB0C-E191FFDF845A</t>
-  </si>
-  <si>
-    <t>56F05333-4945-447A-1128-61D911628D2D</t>
-  </si>
-  <si>
     <t>1B6B8678-D75A-AE62-7CA1-87F8E6BEC7CB</t>
   </si>
   <si>
@@ -886,7 +886,7 @@
     <t>5E11E6A3-7C82-40A3-39DE-32D3F0F53201</t>
   </si>
   <si>
-    <t>lastConection</t>
+    <t>lastConnection</t>
   </si>
   <si>
     <t>80B59BB6-F206-AC15-7CC1-25F0484CB116</t>
@@ -895,19 +895,19 @@
     <t>lastName</t>
   </si>
   <si>
+    <t>0D61A7B9-DD3E-45F7-0461-0E63A231985C</t>
+  </si>
+  <si>
     <t>F987AE6E-E6CD-09F8-BF70-BE0B6F44F316</t>
   </si>
   <si>
-    <t>0D61A7B9-DD3E-45F7-0461-0E63A231985C</t>
-  </si>
-  <si>
     <t>5E39503B-23B3-C4BC-AF2D-6D85A3F3CAB4</t>
   </si>
   <si>
+    <t>30BDE08B-6525-28F3-CF81-72CBF76C81D0</t>
+  </si>
+  <si>
     <t>FD10B671-C4FD-3C2C-5BF2-EC91B141B9E3</t>
-  </si>
-  <si>
-    <t>30BDE08B-6525-28F3-CF81-72CBF76C81D0</t>
   </si>
   <si>
     <t>D1671859-BB90-F668-54B8-2F6B02EEAD4A</t>

</xml_diff>